<commit_message>
Execute Inventory test cases and refine wording
</commit_message>
<xml_diff>
--- a/Test-Cases/Test-Cases-Inventory.xlsx
+++ b/Test-Cases/Test-Cases-Inventory.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\0. Documentos\Github\qa-saucedemo-testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{370A7D98-F80C-40F4-8361-77ABB03D1A0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C235329-6838-499D-BFC1-C976372D23CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-75" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="57">
   <si>
     <t>ID</t>
   </si>
@@ -63,20 +63,9 @@
     <t>Medium</t>
   </si>
   <si>
-    <t>Given the user logged in with standard_user and is on the inventory page
-When they select the "Price (low to high)" option in the sort dropdown
-Then the products are reordered showing the lowest price first, in ascending order</t>
-  </si>
-  <si>
-    <t>Pending</t>
-  </si>
-  <si>
     <t>TC-002</t>
   </si>
   <si>
-    <t>Sort dropdown only responds to clicks on the text, not the arrow icon</t>
-  </si>
-  <si>
     <t>Edge case</t>
   </si>
   <si>
@@ -95,77 +84,40 @@
     <t>High</t>
   </si>
   <si>
-    <t>Given the user is on the inventory page
-When they click the "Add to cart" button on the "Sauce Labs Backpack" product
-Then the button changes to "Remove"
-And the cart icon displays the number "1"</t>
-  </si>
-  <si>
     <t>TC-004</t>
   </si>
   <si>
     <t>Remove a product from the cart via the inventory page</t>
   </si>
   <si>
-    <t>Given the user has a product added to the cart from the inventory page
-When they click the "Remove" button for that product
-Then the button changes back to "Add to cart"
-And the cart counter updates, subtracting that product</t>
-  </si>
-  <si>
     <t>TC-005</t>
   </si>
   <si>
     <t>Add multiple products and verify the cart counter updates correctly</t>
   </si>
   <si>
-    <t>Given the user is on the inventory page
-When they add several products to the cart one by one
-Then the cart icon counter updates correctly after each addition, reflecting the exact quantity</t>
-  </si>
-  <si>
     <t>Pass</t>
   </si>
   <si>
     <t>TC-006</t>
   </si>
   <si>
-    <t>Reset App State does not revert the visual state of the buttons</t>
-  </si>
-  <si>
     <t>TC-007</t>
   </si>
   <si>
     <t>View product detail and return to inventory without losing cart items</t>
   </si>
   <si>
-    <t>Given the user has products added to the cart
-When they click on a product name to view its detail page
-And they return to the inventory page
-Then the previously added products remain in the cart, unaffected</t>
-  </si>
-  <si>
     <t>TC-008</t>
   </si>
   <si>
     <t>Direct access to inventory without an active session</t>
   </si>
   <si>
-    <t>Edge case / Security</t>
-  </si>
-  <si>
-    <t>Given the user does not have an active session
-When they manually enter the URL "https://www.saucedemo.com/inventory.html"
-Then the system displays the message "Epic sadface: You can only access '/inventory.html' when you are logged in." and blocks access to the inventory page</t>
-  </si>
-  <si>
     <t>TC-009</t>
   </si>
   <si>
     <t>TC-010</t>
-  </si>
-  <si>
-    <t>'Item not found'' page displays unrelated placeholder content</t>
   </si>
   <si>
     <t>Negative</t>
@@ -174,15 +126,6 @@
     <t>Given the user is logged in and on the inventory page
 When they manually navigate to a product URL with a non-existent ID (e.g. "https://www.saucedemo.com/inventory-item.html?id=7")
 Then the system should display a clear, relevant "item not found" message</t>
-  </si>
-  <si>
-    <t>Adding a non-existent product to the cart breaks the cart page</t>
-  </si>
-  <si>
-    <t>Given the user is on the "Item not found" page for a non-existent product ID
-When they click "Add to cart"
-And they navigate to the cart view
-Then the system should either prevent adding a non-existent item, or display the cart normally</t>
   </si>
   <si>
     <t>Given the user is on the inventory page
@@ -207,16 +150,79 @@
     <t>Cart counter resets to 0, but the "Remove" buttons don't revert to "Add to cart", visual inconsistency.</t>
   </si>
   <si>
-    <t>Cart contents remain unaffected after viewing a product detail and returning.</t>
-  </si>
-  <si>
     <t>Direct URL access is blocked with a clear error message.</t>
   </si>
   <si>
     <t>"Item not found" page shows unrelated placeholder text (a phone-call message and a stray "$√-1" string) instead of a relevant error.</t>
   </si>
   <si>
-    <t>Adding the non-existent product is allowed, and the cart view then renders completely blank with no error or recovery option.</t>
+    <t>Reset App State reverts the cart counter and the button labels</t>
+  </si>
+  <si>
+    <t>Sort dropdown expands when clicking the text or the arrow icon</t>
+  </si>
+  <si>
+    <t>Given the user has products added to the cart
+When they click on a product name to view its detail page
+And they return to the inventory page using each of these options, one at a time: the "Back to products" option and the browser's back arrow
+Then in both cases the system should return to the inventory page with the previously added products still in the cart</t>
+  </si>
+  <si>
+    <t>Cart contents remain unaffected when returning with the "Back to products" option and with the browser's back arrow.</t>
+  </si>
+  <si>
+    <t>“Item not found” page for a non-existent product ID</t>
+  </si>
+  <si>
+    <t>Add a non-existent product to the cart</t>
+  </si>
+  <si>
+    <t>Given the user is on the "Item not found" page for a non-existent product ID
+When they click "Add to cart"
+And they navigate to the cart view
+Then the system should not allow adding the non-existent product, so the cart counter should not increase and the cart should open normally</t>
+  </si>
+  <si>
+    <t>The system allows adding the non-existent product (cart counter shows 1), but the cart opens empty.</t>
+  </si>
+  <si>
+    <t>The products are reordered with the lowest price first, in ascending order.</t>
+  </si>
+  <si>
+    <t>The button changes to "Remove" and the cart icon displays "1".</t>
+  </si>
+  <si>
+    <t>The button changes back to "Add to cart" and the cart counter updates, subtracting the product.</t>
+  </si>
+  <si>
+    <t>Given the user is logged in with standard_user and is on the inventory page
+When they select the "Price (low to high)" option in the sort dropdown
+Then the products should be reordered, showing the lowest price first, in ascending order</t>
+  </si>
+  <si>
+    <t>Given the user is on the inventory page
+When they click the "Add to cart" button on the "Sauce Labs Backpack" product
+Then the button should change to "Remove"
+And the cart icon should display the number "1"</t>
+  </si>
+  <si>
+    <t>Given the user has a product added to the cart from the inventory page
+When they click the "Remove" button for that product
+Then the button should change back to "Add to cart"
+And the cart counter should update, subtracting that product</t>
+  </si>
+  <si>
+    <t>Given the user is on the inventory page
+When they add several products to the cart one by one
+Then the cart icon counter should update correctly after each addition, reflecting the exact quantity</t>
+  </si>
+  <si>
+    <t>Given the user does not have an active session
+When they manually enter the URL "https://www.saucedemo.com/inventory.html"
+Then the system should display the message "Epic sadface: You can only access '/inventory.html' when you are logged in." and block access to the inventory page</t>
+  </si>
+  <si>
+    <t>Negative / Security</t>
   </si>
 </sst>
 </file>
@@ -320,7 +326,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -349,6 +355,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -623,7 +633,7 @@
     <col min="5" max="5" width="70" customWidth="1"/>
     <col min="6" max="6" width="45" customWidth="1"/>
     <col min="7" max="7" width="12" customWidth="1"/>
-    <col min="8" max="8" width="14" customWidth="1"/>
+    <col min="8" max="8" width="14" style="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -648,11 +658,11 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="10" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
@@ -666,66 +676,76 @@
         <v>11</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="3"/>
+        <v>51</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>48</v>
+      </c>
       <c r="G2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" s="2"/>
+        <v>23</v>
+      </c>
+      <c r="H2" s="8">
+        <v>46304</v>
+      </c>
     </row>
     <row r="3" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="E3" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H3" s="8"/>
+      <c r="H3" s="8">
+        <v>46304</v>
+      </c>
     </row>
     <row r="4" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" s="3"/>
+        <v>52</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>49</v>
+      </c>
       <c r="G4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H4" s="2"/>
+        <v>23</v>
+      </c>
+      <c r="H4" s="8">
+        <v>46304</v>
+      </c>
     </row>
     <row r="5" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>10</v>
@@ -734,68 +754,76 @@
         <v>11</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="F5" s="3"/>
+        <v>53</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>50</v>
+      </c>
       <c r="G5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H5" s="2"/>
-    </row>
-    <row r="6" spans="1:8" ht="70.8" customHeight="1" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+      <c r="H5" s="8">
+        <v>46304</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="64.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="H6" s="2"/>
+        <v>23</v>
+      </c>
+      <c r="H6" s="8">
+        <v>46304</v>
+      </c>
     </row>
     <row r="7" spans="1:8" ht="91.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>11</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H7" s="2"/>
-    </row>
-    <row r="8" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+      <c r="H7" s="8">
+        <v>46304</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="84.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>10</v>
@@ -804,91 +832,99 @@
         <v>11</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="H8" s="2"/>
+        <v>23</v>
+      </c>
+      <c r="H8" s="8">
+        <v>46304</v>
+      </c>
     </row>
     <row r="9" spans="1:8" ht="61.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>37</v>
+        <v>56</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E9" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="F9" s="3" t="s">
-        <v>52</v>
-      </c>
       <c r="G9" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="H9" s="2"/>
+        <v>23</v>
+      </c>
+      <c r="H9" s="8">
+        <v>46304</v>
+      </c>
     </row>
     <row r="10" spans="1:8" ht="61.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="F10" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B10" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>53</v>
-      </c>
       <c r="G10" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H10" s="2"/>
+        <v>15</v>
+      </c>
+      <c r="H10" s="8">
+        <v>46304</v>
+      </c>
     </row>
     <row r="11" spans="1:8" ht="78.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H11" s="2"/>
+        <v>15</v>
+      </c>
+      <c r="H11" s="8">
+        <v>46304</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
-  <dataValidations count="1">
+  <dataValidations disablePrompts="1" count="1">
     <dataValidation type="list" allowBlank="1" sqref="G2:G9" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Pass,Fail,Blocked,Pending"</formula1>
       <formula2>0</formula2>

</xml_diff>